<commit_message>
docs: prepare public distribution with Apache 2.0 license
</commit_message>
<xml_diff>
--- a/backend/fixtures/sample_customers.xlsx
+++ b/backend/fixtures/sample_customers.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,19 +451,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ΑΒΓ Διανομές Α.Ε.</t>
+          <t>Demo customer 1 (synthetic)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>orders@avg-dianomes.test</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2101234567</t>
-        </is>
-      </c>
+          <t>orders@customer1.test</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>ΕΝΕΡΓΟΣ</t>
@@ -478,19 +474,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Μαρκάκης &amp; Σία Ο.Ε.</t>
+          <t>Demo customer 2 (synthetic)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>info@markakis-foods.test</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2310987654</t>
-        </is>
-      </c>
+          <t>orders@customer2.test</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>ΕΝΕΡΓΟΣ</t>
@@ -505,19 +497,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Εστίαση Βορείου Ελλάδος</t>
+          <t>Demo customer 3 (synthetic)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>supply@estiasi-north.test</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2410555666</t>
-        </is>
-      </c>
+          <t>orders@customer3.test</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>ΕΝΕΡΓΟΣ</t>
@@ -532,19 +520,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Παντοπωλείο Η Γωνιά</t>
+          <t>Demo customer 4 (synthetic)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>gonia@fakemail.test</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2810112233</t>
-        </is>
-      </c>
+          <t>orders@customer4.test</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>ΕΝΕΡΓΟΣ</t>

</xml_diff>

<commit_message>
docs: prepare public distribution with Apache 2.0 license (#7)
</commit_message>
<xml_diff>
--- a/backend/fixtures/sample_customers.xlsx
+++ b/backend/fixtures/sample_customers.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,19 +451,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ΑΒΓ Διανομές Α.Ε.</t>
+          <t>Demo customer 1 (synthetic)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>orders@avg-dianomes.test</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2101234567</t>
-        </is>
-      </c>
+          <t>orders@customer1.test</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>ΕΝΕΡΓΟΣ</t>
@@ -478,19 +474,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Μαρκάκης &amp; Σία Ο.Ε.</t>
+          <t>Demo customer 2 (synthetic)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>info@markakis-foods.test</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2310987654</t>
-        </is>
-      </c>
+          <t>orders@customer2.test</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>ΕΝΕΡΓΟΣ</t>
@@ -505,19 +497,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Εστίαση Βορείου Ελλάδος</t>
+          <t>Demo customer 3 (synthetic)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>supply@estiasi-north.test</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2410555666</t>
-        </is>
-      </c>
+          <t>orders@customer3.test</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>ΕΝΕΡΓΟΣ</t>
@@ -532,19 +520,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Παντοπωλείο Η Γωνιά</t>
+          <t>Demo customer 4 (synthetic)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>gonia@fakemail.test</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2810112233</t>
-        </is>
-      </c>
+          <t>orders@customer4.test</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>ΕΝΕΡΓΟΣ</t>

</xml_diff>